<commit_message>
Changing formatting in APR export; adding dates paste formats
</commit_message>
<xml_diff>
--- a/core/api/export/templates/APRAnnexI.xlsx
+++ b/core/api/export/templates/APRAnnexI.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Annex I APR report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annex I APR report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annex I APR report'!$A$1:$AX$3</definedName>
@@ -14,11 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="[$-409]mmm/yy"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="[$-409]DD-MMM-YY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -104,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -171,6 +172,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -776,10 +780,10 @@
           <t>Extension of institutional strengthening project (phase X: 1/2022-12/2023)</t>
         </is>
       </c>
-      <c r="K2" s="15" t="n">
+      <c r="K2" s="28" t="n">
         <v>45627</v>
       </c>
-      <c r="L2" s="15" t="n">
+      <c r="L2" s="28" t="n">
         <v>46722</v>
       </c>
       <c r="M2" s="14" t="inlineStr">
@@ -787,10 +791,10 @@
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="N2" s="15" t="n"/>
-      <c r="O2" s="15" t="n"/>
-      <c r="P2" s="15" t="n"/>
-      <c r="Q2" s="15" t="n"/>
+      <c r="N2" s="28" t="n"/>
+      <c r="O2" s="28" t="n"/>
+      <c r="P2" s="28" t="n"/>
+      <c r="Q2" s="28" t="n"/>
       <c r="R2" s="16" t="n"/>
       <c r="S2" s="16" t="n"/>
       <c r="T2" s="17" t="n"/>
@@ -803,36 +807,36 @@
       <c r="AA2" s="18" t="n"/>
       <c r="AB2" s="18" t="n"/>
       <c r="AC2" s="18" t="n"/>
-      <c r="AD2" s="19" t="n">
+      <c r="AD2" s="18" t="n">
         <v>192000</v>
       </c>
-      <c r="AE2" s="19" t="n"/>
-      <c r="AF2" s="19" t="n">
+      <c r="AE2" s="18" t="n"/>
+      <c r="AF2" s="18" t="n">
         <v>192000</v>
       </c>
       <c r="AG2" s="19" t="n"/>
-      <c r="AH2" s="19" t="n">
+      <c r="AH2" s="18" t="n">
         <v>192000</v>
       </c>
-      <c r="AI2" s="19" t="n">
+      <c r="AI2" s="18" t="n">
         <v>13440</v>
       </c>
-      <c r="AJ2" s="19" t="n"/>
-      <c r="AK2" s="19" t="n">
+      <c r="AJ2" s="18" t="n"/>
+      <c r="AK2" s="18" t="n">
         <v>13440</v>
       </c>
-      <c r="AL2" s="19" t="n">
+      <c r="AL2" s="18" t="n">
         <v>13440</v>
       </c>
-      <c r="AM2" s="19" t="n"/>
-      <c r="AN2" s="19" t="n"/>
-      <c r="AO2" s="19" t="n"/>
-      <c r="AP2" s="19" t="n"/>
-      <c r="AQ2" s="19" t="n"/>
-      <c r="AR2" s="19" t="n"/>
-      <c r="AS2" s="19" t="n"/>
+      <c r="AM2" s="18" t="n"/>
+      <c r="AN2" s="18" t="n"/>
+      <c r="AO2" s="18" t="n"/>
+      <c r="AP2" s="18" t="n"/>
+      <c r="AQ2" s="18" t="n"/>
+      <c r="AR2" s="18" t="n"/>
+      <c r="AS2" s="18" t="n"/>
       <c r="AT2" s="20" t="n"/>
-      <c r="AU2" s="15" t="n">
+      <c r="AU2" s="28" t="n">
         <v>46722</v>
       </c>
       <c r="AV2" s="20" t="n"/>
@@ -894,10 +898,10 @@
           <t>Preparation of national inventory of banks of waste-controlled substances and development of a national plan for management of these substances (decision 91/66)</t>
         </is>
       </c>
-      <c r="K3" s="15" t="n">
+      <c r="K3" s="28" t="n">
         <v>45413</v>
       </c>
-      <c r="L3" s="15" t="n">
+      <c r="L3" s="28" t="n">
         <v>46174</v>
       </c>
       <c r="M3" s="14" t="inlineStr">
@@ -905,10 +909,10 @@
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="N3" s="15" t="n"/>
-      <c r="O3" s="15" t="n"/>
-      <c r="P3" s="15" t="n"/>
-      <c r="Q3" s="15" t="n"/>
+      <c r="N3" s="28" t="n"/>
+      <c r="O3" s="28" t="n"/>
+      <c r="P3" s="28" t="n"/>
+      <c r="Q3" s="28" t="n"/>
       <c r="R3" s="16" t="n"/>
       <c r="S3" s="16" t="n"/>
       <c r="T3" s="17" t="n"/>
@@ -921,36 +925,36 @@
       <c r="AA3" s="18" t="n"/>
       <c r="AB3" s="18" t="n"/>
       <c r="AC3" s="18" t="n"/>
-      <c r="AD3" s="19" t="n">
+      <c r="AD3" s="18" t="n">
         <v>90000</v>
       </c>
-      <c r="AE3" s="19" t="n"/>
-      <c r="AF3" s="19" t="n">
+      <c r="AE3" s="18" t="n"/>
+      <c r="AF3" s="18" t="n">
         <v>90000</v>
       </c>
       <c r="AG3" s="19" t="n"/>
-      <c r="AH3" s="19" t="n">
+      <c r="AH3" s="18" t="n">
         <v>90000</v>
       </c>
-      <c r="AI3" s="19" t="n">
+      <c r="AI3" s="18" t="n">
         <v>6300</v>
       </c>
-      <c r="AJ3" s="19" t="n"/>
-      <c r="AK3" s="19" t="n">
+      <c r="AJ3" s="18" t="n"/>
+      <c r="AK3" s="18" t="n">
         <v>6300</v>
       </c>
-      <c r="AL3" s="19" t="n">
+      <c r="AL3" s="18" t="n">
         <v>6300</v>
       </c>
-      <c r="AM3" s="19" t="n"/>
-      <c r="AN3" s="19" t="n"/>
-      <c r="AO3" s="19" t="n"/>
-      <c r="AP3" s="19" t="n"/>
-      <c r="AQ3" s="19" t="n"/>
-      <c r="AR3" s="19" t="n"/>
-      <c r="AS3" s="19" t="n"/>
+      <c r="AM3" s="18" t="n"/>
+      <c r="AN3" s="18" t="n"/>
+      <c r="AO3" s="18" t="n"/>
+      <c r="AP3" s="18" t="n"/>
+      <c r="AQ3" s="18" t="n"/>
+      <c r="AR3" s="18" t="n"/>
+      <c r="AS3" s="18" t="n"/>
       <c r="AT3" s="20" t="n"/>
-      <c r="AU3" s="15" t="n">
+      <c r="AU3" s="28" t="n">
         <v>46174</v>
       </c>
       <c r="AV3" s="20" t="n"/>

</xml_diff>

<commit_message>
Changing formatting in APR export; adding dates paste formats (#1193)
</commit_message>
<xml_diff>
--- a/core/api/export/templates/APRAnnexI.xlsx
+++ b/core/api/export/templates/APRAnnexI.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Annex I APR report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annex I APR report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annex I APR report'!$A$1:$AX$3</definedName>
@@ -14,11 +14,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="[$-409]mmm/yy"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
+    <numFmt numFmtId="168" formatCode="[$-409]DD-MMM-YY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -104,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -171,6 +172,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -776,10 +780,10 @@
           <t>Extension of institutional strengthening project (phase X: 1/2022-12/2023)</t>
         </is>
       </c>
-      <c r="K2" s="15" t="n">
+      <c r="K2" s="28" t="n">
         <v>45627</v>
       </c>
-      <c r="L2" s="15" t="n">
+      <c r="L2" s="28" t="n">
         <v>46722</v>
       </c>
       <c r="M2" s="14" t="inlineStr">
@@ -787,10 +791,10 @@
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="N2" s="15" t="n"/>
-      <c r="O2" s="15" t="n"/>
-      <c r="P2" s="15" t="n"/>
-      <c r="Q2" s="15" t="n"/>
+      <c r="N2" s="28" t="n"/>
+      <c r="O2" s="28" t="n"/>
+      <c r="P2" s="28" t="n"/>
+      <c r="Q2" s="28" t="n"/>
       <c r="R2" s="16" t="n"/>
       <c r="S2" s="16" t="n"/>
       <c r="T2" s="17" t="n"/>
@@ -803,36 +807,36 @@
       <c r="AA2" s="18" t="n"/>
       <c r="AB2" s="18" t="n"/>
       <c r="AC2" s="18" t="n"/>
-      <c r="AD2" s="19" t="n">
+      <c r="AD2" s="18" t="n">
         <v>192000</v>
       </c>
-      <c r="AE2" s="19" t="n"/>
-      <c r="AF2" s="19" t="n">
+      <c r="AE2" s="18" t="n"/>
+      <c r="AF2" s="18" t="n">
         <v>192000</v>
       </c>
       <c r="AG2" s="19" t="n"/>
-      <c r="AH2" s="19" t="n">
+      <c r="AH2" s="18" t="n">
         <v>192000</v>
       </c>
-      <c r="AI2" s="19" t="n">
+      <c r="AI2" s="18" t="n">
         <v>13440</v>
       </c>
-      <c r="AJ2" s="19" t="n"/>
-      <c r="AK2" s="19" t="n">
+      <c r="AJ2" s="18" t="n"/>
+      <c r="AK2" s="18" t="n">
         <v>13440</v>
       </c>
-      <c r="AL2" s="19" t="n">
+      <c r="AL2" s="18" t="n">
         <v>13440</v>
       </c>
-      <c r="AM2" s="19" t="n"/>
-      <c r="AN2" s="19" t="n"/>
-      <c r="AO2" s="19" t="n"/>
-      <c r="AP2" s="19" t="n"/>
-      <c r="AQ2" s="19" t="n"/>
-      <c r="AR2" s="19" t="n"/>
-      <c r="AS2" s="19" t="n"/>
+      <c r="AM2" s="18" t="n"/>
+      <c r="AN2" s="18" t="n"/>
+      <c r="AO2" s="18" t="n"/>
+      <c r="AP2" s="18" t="n"/>
+      <c r="AQ2" s="18" t="n"/>
+      <c r="AR2" s="18" t="n"/>
+      <c r="AS2" s="18" t="n"/>
       <c r="AT2" s="20" t="n"/>
-      <c r="AU2" s="15" t="n">
+      <c r="AU2" s="28" t="n">
         <v>46722</v>
       </c>
       <c r="AV2" s="20" t="n"/>
@@ -894,10 +898,10 @@
           <t>Preparation of national inventory of banks of waste-controlled substances and development of a national plan for management of these substances (decision 91/66)</t>
         </is>
       </c>
-      <c r="K3" s="15" t="n">
+      <c r="K3" s="28" t="n">
         <v>45413</v>
       </c>
-      <c r="L3" s="15" t="n">
+      <c r="L3" s="28" t="n">
         <v>46174</v>
       </c>
       <c r="M3" s="14" t="inlineStr">
@@ -905,10 +909,10 @@
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="N3" s="15" t="n"/>
-      <c r="O3" s="15" t="n"/>
-      <c r="P3" s="15" t="n"/>
-      <c r="Q3" s="15" t="n"/>
+      <c r="N3" s="28" t="n"/>
+      <c r="O3" s="28" t="n"/>
+      <c r="P3" s="28" t="n"/>
+      <c r="Q3" s="28" t="n"/>
       <c r="R3" s="16" t="n"/>
       <c r="S3" s="16" t="n"/>
       <c r="T3" s="17" t="n"/>
@@ -921,36 +925,36 @@
       <c r="AA3" s="18" t="n"/>
       <c r="AB3" s="18" t="n"/>
       <c r="AC3" s="18" t="n"/>
-      <c r="AD3" s="19" t="n">
+      <c r="AD3" s="18" t="n">
         <v>90000</v>
       </c>
-      <c r="AE3" s="19" t="n"/>
-      <c r="AF3" s="19" t="n">
+      <c r="AE3" s="18" t="n"/>
+      <c r="AF3" s="18" t="n">
         <v>90000</v>
       </c>
       <c r="AG3" s="19" t="n"/>
-      <c r="AH3" s="19" t="n">
+      <c r="AH3" s="18" t="n">
         <v>90000</v>
       </c>
-      <c r="AI3" s="19" t="n">
+      <c r="AI3" s="18" t="n">
         <v>6300</v>
       </c>
-      <c r="AJ3" s="19" t="n"/>
-      <c r="AK3" s="19" t="n">
+      <c r="AJ3" s="18" t="n"/>
+      <c r="AK3" s="18" t="n">
         <v>6300</v>
       </c>
-      <c r="AL3" s="19" t="n">
+      <c r="AL3" s="18" t="n">
         <v>6300</v>
       </c>
-      <c r="AM3" s="19" t="n"/>
-      <c r="AN3" s="19" t="n"/>
-      <c r="AO3" s="19" t="n"/>
-      <c r="AP3" s="19" t="n"/>
-      <c r="AQ3" s="19" t="n"/>
-      <c r="AR3" s="19" t="n"/>
-      <c r="AS3" s="19" t="n"/>
+      <c r="AM3" s="18" t="n"/>
+      <c r="AN3" s="18" t="n"/>
+      <c r="AO3" s="18" t="n"/>
+      <c r="AP3" s="18" t="n"/>
+      <c r="AQ3" s="18" t="n"/>
+      <c r="AR3" s="18" t="n"/>
+      <c r="AS3" s="18" t="n"/>
       <c r="AT3" s="20" t="n"/>
-      <c r="AU3" s="15" t="n">
+      <c r="AU3" s="28" t="n">
         <v>46174</v>
       </c>
       <c r="AV3" s="20" t="n"/>

</xml_diff>

<commit_message>
Revert "Changing formatting in APR export; adding dates paste formats (#1193)"
This reverts commit c797e9dd7a83da16267c257c634c9a00d6cc1b43.

The MLF realized it will hamper their work; they'll want this back in Nov 2026
</commit_message>
<xml_diff>
--- a/core/api/export/templates/APRAnnexI.xlsx
+++ b/core/api/export/templates/APRAnnexI.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annex I APR report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Annex I APR report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annex I APR report'!$A$1:$AX$3</definedName>
@@ -14,12 +14,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="[$-409]mmm/yy"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@"/>
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
-    <numFmt numFmtId="168" formatCode="[$-409]DD-MMM-YY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -105,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -172,9 +171,6 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -780,10 +776,10 @@
           <t>Extension of institutional strengthening project (phase X: 1/2022-12/2023)</t>
         </is>
       </c>
-      <c r="K2" s="28" t="n">
+      <c r="K2" s="15" t="n">
         <v>45627</v>
       </c>
-      <c r="L2" s="28" t="n">
+      <c r="L2" s="15" t="n">
         <v>46722</v>
       </c>
       <c r="M2" s="14" t="inlineStr">
@@ -791,10 +787,10 @@
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="N2" s="28" t="n"/>
-      <c r="O2" s="28" t="n"/>
-      <c r="P2" s="28" t="n"/>
-      <c r="Q2" s="28" t="n"/>
+      <c r="N2" s="15" t="n"/>
+      <c r="O2" s="15" t="n"/>
+      <c r="P2" s="15" t="n"/>
+      <c r="Q2" s="15" t="n"/>
       <c r="R2" s="16" t="n"/>
       <c r="S2" s="16" t="n"/>
       <c r="T2" s="17" t="n"/>
@@ -807,36 +803,36 @@
       <c r="AA2" s="18" t="n"/>
       <c r="AB2" s="18" t="n"/>
       <c r="AC2" s="18" t="n"/>
-      <c r="AD2" s="18" t="n">
+      <c r="AD2" s="19" t="n">
         <v>192000</v>
       </c>
-      <c r="AE2" s="18" t="n"/>
-      <c r="AF2" s="18" t="n">
+      <c r="AE2" s="19" t="n"/>
+      <c r="AF2" s="19" t="n">
         <v>192000</v>
       </c>
       <c r="AG2" s="19" t="n"/>
-      <c r="AH2" s="18" t="n">
+      <c r="AH2" s="19" t="n">
         <v>192000</v>
       </c>
-      <c r="AI2" s="18" t="n">
+      <c r="AI2" s="19" t="n">
         <v>13440</v>
       </c>
-      <c r="AJ2" s="18" t="n"/>
-      <c r="AK2" s="18" t="n">
+      <c r="AJ2" s="19" t="n"/>
+      <c r="AK2" s="19" t="n">
         <v>13440</v>
       </c>
-      <c r="AL2" s="18" t="n">
+      <c r="AL2" s="19" t="n">
         <v>13440</v>
       </c>
-      <c r="AM2" s="18" t="n"/>
-      <c r="AN2" s="18" t="n"/>
-      <c r="AO2" s="18" t="n"/>
-      <c r="AP2" s="18" t="n"/>
-      <c r="AQ2" s="18" t="n"/>
-      <c r="AR2" s="18" t="n"/>
-      <c r="AS2" s="18" t="n"/>
+      <c r="AM2" s="19" t="n"/>
+      <c r="AN2" s="19" t="n"/>
+      <c r="AO2" s="19" t="n"/>
+      <c r="AP2" s="19" t="n"/>
+      <c r="AQ2" s="19" t="n"/>
+      <c r="AR2" s="19" t="n"/>
+      <c r="AS2" s="19" t="n"/>
       <c r="AT2" s="20" t="n"/>
-      <c r="AU2" s="28" t="n">
+      <c r="AU2" s="15" t="n">
         <v>46722</v>
       </c>
       <c r="AV2" s="20" t="n"/>
@@ -898,10 +894,10 @@
           <t>Preparation of national inventory of banks of waste-controlled substances and development of a national plan for management of these substances (decision 91/66)</t>
         </is>
       </c>
-      <c r="K3" s="28" t="n">
+      <c r="K3" s="15" t="n">
         <v>45413</v>
       </c>
-      <c r="L3" s="28" t="n">
+      <c r="L3" s="15" t="n">
         <v>46174</v>
       </c>
       <c r="M3" s="14" t="inlineStr">
@@ -909,10 +905,10 @@
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="N3" s="28" t="n"/>
-      <c r="O3" s="28" t="n"/>
-      <c r="P3" s="28" t="n"/>
-      <c r="Q3" s="28" t="n"/>
+      <c r="N3" s="15" t="n"/>
+      <c r="O3" s="15" t="n"/>
+      <c r="P3" s="15" t="n"/>
+      <c r="Q3" s="15" t="n"/>
       <c r="R3" s="16" t="n"/>
       <c r="S3" s="16" t="n"/>
       <c r="T3" s="17" t="n"/>
@@ -925,36 +921,36 @@
       <c r="AA3" s="18" t="n"/>
       <c r="AB3" s="18" t="n"/>
       <c r="AC3" s="18" t="n"/>
-      <c r="AD3" s="18" t="n">
+      <c r="AD3" s="19" t="n">
         <v>90000</v>
       </c>
-      <c r="AE3" s="18" t="n"/>
-      <c r="AF3" s="18" t="n">
+      <c r="AE3" s="19" t="n"/>
+      <c r="AF3" s="19" t="n">
         <v>90000</v>
       </c>
       <c r="AG3" s="19" t="n"/>
-      <c r="AH3" s="18" t="n">
+      <c r="AH3" s="19" t="n">
         <v>90000</v>
       </c>
-      <c r="AI3" s="18" t="n">
+      <c r="AI3" s="19" t="n">
         <v>6300</v>
       </c>
-      <c r="AJ3" s="18" t="n"/>
-      <c r="AK3" s="18" t="n">
+      <c r="AJ3" s="19" t="n"/>
+      <c r="AK3" s="19" t="n">
         <v>6300</v>
       </c>
-      <c r="AL3" s="18" t="n">
+      <c r="AL3" s="19" t="n">
         <v>6300</v>
       </c>
-      <c r="AM3" s="18" t="n"/>
-      <c r="AN3" s="18" t="n"/>
-      <c r="AO3" s="18" t="n"/>
-      <c r="AP3" s="18" t="n"/>
-      <c r="AQ3" s="18" t="n"/>
-      <c r="AR3" s="18" t="n"/>
-      <c r="AS3" s="18" t="n"/>
+      <c r="AM3" s="19" t="n"/>
+      <c r="AN3" s="19" t="n"/>
+      <c r="AO3" s="19" t="n"/>
+      <c r="AP3" s="19" t="n"/>
+      <c r="AQ3" s="19" t="n"/>
+      <c r="AR3" s="19" t="n"/>
+      <c r="AS3" s="19" t="n"/>
       <c r="AT3" s="20" t="n"/>
-      <c r="AU3" s="28" t="n">
+      <c r="AU3" s="15" t="n">
         <v>46174</v>
       </c>
       <c r="AV3" s="20" t="n"/>

</xml_diff>